<commit_message>
Did a balance for Birkett, updated some numbers
</commit_message>
<xml_diff>
--- a/mill_floor.xlsx
+++ b/mill_floor.xlsx
@@ -262,10 +262,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="13863637" cy="4095750"/>
+    <ext cx="7178039" cy="2120616"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -573,18 +573,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -617,7 +617,7 @@
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CANE FEED</t>
+          <t>PROCESS FLOW DIAGRAM</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -627,250 +627,42 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Cane throughput</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>17000</v>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>TPD</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Cane pol</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Cane fiber</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Imbibition</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>% on cane</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Imbibition flow</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>711.178045515395</v>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>GPM</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>MIXED JUICE</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>1361898.625429553</v>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Brix</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>15.34365098708262</v>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Purity</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>88</v>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Pol</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="n">
-        <v>13.50241286863271</v>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n">
-        <v>90</v>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>°F</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>2566.951420420189</v>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>GPM</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>BAGASSE</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>408934.70790378</v>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n">
-        <v>4907.216494845361</v>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>TPD</t>
-        </is>
-      </c>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>CANE FEED</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Fiber</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>48.5</v>
+          <t>Cane throughput</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>17000</v>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>TPD</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Pol</t>
+          <t>Cane pol</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>1.8</v>
+        <v>13.5</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
@@ -881,11 +673,11 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Brix</t>
+          <t>Cane fiber</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>2.5</v>
+        <v>14</v>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
@@ -896,511 +688,723 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>Imbibition</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>% on cane</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Imbibition flow</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>711.178045515395</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>GPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MIXED JUICE</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>1361898.625429553</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Brix</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>15.34365098708262</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Purity</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Pol</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>13.50241286863271</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>2566.951420420189</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>GPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>BAGASSE</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>408934.70790378</v>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>4907.216494845361</v>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>TPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Fiber</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Pol</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Brix</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
           <t>Moisture</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n">
+      <c r="B43" s="9" t="n">
         <v>49</v>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="45" ht="17" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>PERFORMANCE</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>Mill extraction</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B46" s="9" t="n">
         <v>96.15120274914088</v>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>% pol in cane</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="48" ht="17" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>STREAM TABLE  (TPH)</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>Dir</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>Flow (TPH)</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Pol (TPH)</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>Brix (TPH)</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr">
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t>Fiber (TPH)</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>Water (TPH)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t>Cane</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C33" s="13" t="n">
+      <c r="C50" s="13" t="n">
         <v>708.3333333333334</v>
       </c>
-      <c r="D33" s="13" t="n">
+      <c r="D50" s="13" t="n">
         <v>95.625</v>
       </c>
-      <c r="E33" s="13" t="n">
+      <c r="E50" s="13" t="n">
         <v>109.5941697906904</v>
       </c>
-      <c r="F33" s="13" t="n">
+      <c r="F50" s="13" t="n">
         <v>99.16666666666669</v>
       </c>
-      <c r="G33" s="13" t="n">
+      <c r="G50" s="13" t="n">
         <v>499.5724968759763</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>Imbibition</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C34" s="15" t="n">
+      <c r="C51" s="15" t="n">
         <v>177.0833333333333</v>
       </c>
-      <c r="D34" s="15" t="n">
+      <c r="D51" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="15" t="n">
+      <c r="E51" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="15" t="n">
+      <c r="F51" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="15" t="n">
+      <c r="G51" s="15" t="n">
         <v>177.0833333333333</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>Mixed Juice</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
+      <c r="C52" s="13" t="n">
         <v>680.9493127147766</v>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D52" s="13" t="n">
         <v>91.94458762886596</v>
       </c>
-      <c r="E35" s="13" t="n">
+      <c r="E52" s="13" t="n">
         <v>104.4824859418932</v>
       </c>
-      <c r="F35" s="13" t="n">
+      <c r="F52" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="13" t="n">
+      <c r="G52" s="13" t="n">
         <v>576.4668267728835</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>Bagasse</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C36" s="15" t="n">
+      <c r="C53" s="15" t="n">
         <v>204.46735395189</v>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D53" s="15" t="n">
         <v>3.680412371134021</v>
       </c>
-      <c r="E36" s="15" t="n">
+      <c r="E53" s="15" t="n">
         <v>5.11168384879725</v>
       </c>
-      <c r="F36" s="15" t="n">
+      <c r="F53" s="15" t="n">
         <v>99.16666666666666</v>
       </c>
-      <c r="G36" s="15" t="n">
+      <c r="G53" s="15" t="n">
         <v>100.1890034364261</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>Total In</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr"/>
-      <c r="C37" s="17" t="n">
+      <c r="B54" s="16" t="inlineStr"/>
+      <c r="C54" s="17" t="n">
         <v>885.4166666666667</v>
       </c>
-      <c r="D37" s="17" t="n">
+      <c r="D54" s="17" t="n">
         <v>95.625</v>
       </c>
-      <c r="E37" s="17" t="n">
+      <c r="E54" s="17" t="n">
         <v>109.5941697906904</v>
       </c>
-      <c r="F37" s="17" t="n">
+      <c r="F54" s="17" t="n">
         <v>99.16666666666669</v>
       </c>
-      <c r="G37" s="17" t="n">
+      <c r="G54" s="17" t="n">
         <v>676.6558302093097</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>Total Out</t>
         </is>
       </c>
-      <c r="B38" s="16" t="inlineStr"/>
-      <c r="C38" s="17" t="n">
+      <c r="B55" s="16" t="inlineStr"/>
+      <c r="C55" s="17" t="n">
         <v>885.4166666666666</v>
       </c>
-      <c r="D38" s="17" t="n">
+      <c r="D55" s="17" t="n">
         <v>95.62499999999999</v>
       </c>
-      <c r="E38" s="17" t="n">
+      <c r="E55" s="17" t="n">
         <v>109.5941697906904</v>
       </c>
-      <c r="F38" s="17" t="n">
+      <c r="F55" s="17" t="n">
         <v>99.16666666666666</v>
       </c>
-      <c r="G38" s="17" t="n">
+      <c r="G55" s="17" t="n">
         <v>676.6558302093096</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
-      <c r="B39" s="16" t="inlineStr"/>
-      <c r="C39" s="17" t="n">
+      <c r="B56" s="16" t="inlineStr"/>
+      <c r="C56" s="17" t="n">
         <v>1.13686837721616e-13</v>
       </c>
-      <c r="D39" s="17" t="n">
+      <c r="D56" s="17" t="n">
         <v>1.4210854715202e-14</v>
       </c>
-      <c r="E39" s="17" t="n">
+      <c r="E56" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="17" t="n">
+      <c r="F56" s="17" t="n">
         <v>2.842170943040401e-14</v>
       </c>
-      <c r="G39" s="17" t="n">
+      <c r="G56" s="17" t="n">
         <v>1.13686837721616e-13</v>
       </c>
     </row>
-    <row r="41" ht="17" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>PER-MILL MACERATION BALANCE  (TPD)</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="5" t="n"/>
+      <c r="F58" s="5" t="n"/>
+      <c r="G58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>Mill</t>
         </is>
       </c>
-      <c r="B42" s="11" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>Bagasse In</t>
         </is>
       </c>
-      <c r="C42" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Liquid In</t>
         </is>
       </c>
-      <c r="D42" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Liquid In Source</t>
         </is>
       </c>
-      <c r="E42" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Bagasse Out</t>
         </is>
       </c>
-      <c r="F42" s="11" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Juice Out</t>
         </is>
       </c>
-      <c r="G42" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>Juice Out Dest</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="18" t="n">
+    <row r="60">
+      <c r="A60" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B43" s="19" t="n">
+      <c r="B60" s="19" t="n">
         <v>17000</v>
       </c>
-      <c r="C43" s="19" t="n">
+      <c r="C60" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E43" s="19" t="n">
+      <c r="E60" s="19" t="n">
         <v>9127.51677852349</v>
       </c>
-      <c r="F43" s="19" t="n">
+      <c r="F60" s="19" t="n">
         <v>7872.48322147651</v>
       </c>
-      <c r="G43" s="12" t="inlineStr">
+      <c r="G60" s="12" t="inlineStr">
         <is>
           <t>To process</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="20" t="n">
+    <row r="61">
+      <c r="A61" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B44" s="21" t="n">
+      <c r="B61" s="21" t="n">
         <v>9127.51677852349</v>
       </c>
-      <c r="C44" s="21" t="n">
+      <c r="C61" s="21" t="n">
         <v>7130.741620337885</v>
       </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>Mill 3 maceration</t>
         </is>
       </c>
-      <c r="E44" s="21" t="n">
+      <c r="E61" s="21" t="n">
         <v>7787.958115183246</v>
       </c>
-      <c r="F44" s="21" t="n">
+      <c r="F61" s="21" t="n">
         <v>8470.300283678129</v>
       </c>
-      <c r="G44" s="14" t="inlineStr">
+      <c r="G61" s="14" t="inlineStr">
         <is>
           <t>To process</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="18" t="n">
+    <row r="62">
+      <c r="A62" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B45" s="19" t="n">
+      <c r="B62" s="19" t="n">
         <v>7787.958115183246</v>
       </c>
-      <c r="C45" s="19" t="n">
+      <c r="C62" s="19" t="n">
         <v>6134.051874394188</v>
       </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>Mill 4 maceration</t>
         </is>
       </c>
-      <c r="E45" s="19" t="n">
+      <c r="E62" s="19" t="n">
         <v>6791.268369239549</v>
       </c>
-      <c r="F45" s="19" t="n">
+      <c r="F62" s="19" t="n">
         <v>7130.741620337885</v>
       </c>
-      <c r="G45" s="12" t="inlineStr">
+      <c r="G62" s="12" t="inlineStr">
         <is>
           <t>Mill 2 maceration</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="20" t="n">
+    <row r="63">
+      <c r="A63" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B46" s="21" t="n">
+      <c r="B63" s="21" t="n">
         <v>6791.268369239549</v>
       </c>
-      <c r="C46" s="21" t="n">
+      <c r="C63" s="21" t="n">
         <v>5363.527244087096</v>
       </c>
-      <c r="D46" s="14" t="inlineStr">
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>Mill 5 maceration</t>
         </is>
       </c>
-      <c r="E46" s="21" t="n">
+      <c r="E63" s="21" t="n">
         <v>6020.743738932457</v>
       </c>
-      <c r="F46" s="21" t="n">
+      <c r="F63" s="21" t="n">
         <v>6134.051874394188</v>
       </c>
-      <c r="G46" s="14" t="inlineStr">
+      <c r="G63" s="14" t="inlineStr">
         <is>
           <t>Mill 3 maceration</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="18" t="n">
+    <row r="64">
+      <c r="A64" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B47" s="19" t="n">
+      <c r="B64" s="19" t="n">
         <v>6020.743738932457</v>
       </c>
-      <c r="C47" s="19" t="n">
+      <c r="C64" s="19" t="n">
         <v>4750.031034406031</v>
       </c>
-      <c r="D47" s="12" t="inlineStr">
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>Mill 6 maceration</t>
         </is>
       </c>
-      <c r="E47" s="19" t="n">
+      <c r="E64" s="19" t="n">
         <v>5407.247529251392</v>
       </c>
-      <c r="F47" s="19" t="n">
+      <c r="F64" s="19" t="n">
         <v>5363.527244087096</v>
       </c>
-      <c r="G47" s="12" t="inlineStr">
+      <c r="G64" s="12" t="inlineStr">
         <is>
           <t>Mill 4 maceration</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="20" t="n">
+    <row r="65">
+      <c r="A65" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B48" s="21" t="n">
+      <c r="B65" s="21" t="n">
         <v>5407.247529251392</v>
       </c>
-      <c r="C48" s="21" t="n">
+      <c r="C65" s="21" t="n">
         <v>4250</v>
       </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>Imbibition</t>
         </is>
       </c>
-      <c r="E48" s="21" t="n">
+      <c r="E65" s="21" t="n">
         <v>4907.216494845361</v>
       </c>
-      <c r="F48" s="21" t="n">
+      <c r="F65" s="21" t="n">
         <v>4750.031034406031</v>
       </c>
-      <c r="G48" s="14" t="inlineStr">
+      <c r="G65" s="14" t="inlineStr">
         <is>
           <t>Mill 5 maceration</t>
         </is>
       </c>
-    </row>
-    <row r="50" ht="17" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>PROCESS FLOW DIAGRAM</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A48:G48"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="46" min="0" max="16383" man="1"/>
+  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>